<commit_message>
Removed the HLA class I ortholog gene and added the PF4 gene
</commit_message>
<xml_diff>
--- a/data/raw/gene_list/macrophage_associated_proteins.xlsx
+++ b/data/raw/gene_list/macrophage_associated_proteins.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10601"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/giraudmn/Documents/ams gwas/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/endritjakupi/Desktop/cardiovascular-snp-analysis/data/raw/gene_list/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{13D9959A-CEF2-3E48-B79C-55CE9B4D44C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{806939DE-BE04-CA40-9567-F7B7C3B7518C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="70960" yWindow="-780" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Macrophage_protein_table" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="278">
   <si>
     <t>Macrophage-associated proteins identified in the infarcted secretome</t>
   </si>
@@ -834,21 +834,6 @@
     <t>Antigen-presentation component; included as supportive immune biology despite q-value above 0.05.</t>
   </si>
   <si>
-    <t>RT1-Aw2</t>
-  </si>
-  <si>
-    <t>HLA class I ortholog</t>
-  </si>
-  <si>
-    <t>MHC class I antigen, RT1-Aw2</t>
-  </si>
-  <si>
-    <t>Antigen presentation</t>
-  </si>
-  <si>
-    <t>Rat MHC class I protein supporting the antigen-presentation component of the immune signature.</t>
-  </si>
-  <si>
     <t>Notes</t>
   </si>
   <si>
@@ -880,6 +865,9 @@
   </si>
   <si>
     <t>Rows with q-value &gt; 0.05 are labeled Secondary or supportive candidates when biologically relevant.</t>
+  </si>
+  <si>
+    <t>PF4</t>
   </si>
 </sst>
 </file>
@@ -976,7 +964,28 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="6">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1012,7 +1021,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MacrophageProteinTable" displayName="MacrophageProteinTable" ref="A4:K56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="MacrophageProteinTable" displayName="MacrophageProteinTable" ref="A4:K55">
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Rat gene"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Human gene"/>
@@ -2454,14 +2463,14 @@
         <v>174</v>
       </c>
       <c r="D37" s="4" t="str">
-        <f t="shared" ref="D37:D68" si="2">IF(E37&gt;0,"Up",IF(E37&lt;0,"Down","No change"))</f>
+        <f>IF(E37&gt;0,"Up",IF(E37&lt;0,"Down","No change"))</f>
         <v>Up</v>
       </c>
       <c r="E37" s="5">
         <v>1.0720000000000001</v>
       </c>
       <c r="F37" s="5">
-        <f t="shared" ref="F37:F68" si="3">2^E37</f>
+        <f>2^E37</f>
         <v>2.1023458181754129</v>
       </c>
       <c r="G37" s="6">
@@ -2491,14 +2500,14 @@
         <v>179</v>
       </c>
       <c r="D38" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E38&gt;0,"Up",IF(E38&lt;0,"Down","No change"))</f>
         <v>Up</v>
       </c>
       <c r="E38" s="5">
         <v>0.89500000000000002</v>
       </c>
       <c r="F38" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E38</f>
         <v>1.8596098852263236</v>
       </c>
       <c r="G38" s="6">
@@ -2528,14 +2537,14 @@
         <v>184</v>
       </c>
       <c r="D39" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E39&gt;0,"Up",IF(E39&lt;0,"Down","No change"))</f>
         <v>Up</v>
       </c>
       <c r="E39" s="5">
         <v>2.1219999999999999</v>
       </c>
       <c r="F39" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E39</f>
         <v>4.3529697666832146</v>
       </c>
       <c r="G39" s="6">
@@ -2565,14 +2574,14 @@
         <v>189</v>
       </c>
       <c r="D40" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E40&gt;0,"Up",IF(E40&lt;0,"Down","No change"))</f>
         <v>Up</v>
       </c>
       <c r="E40" s="5">
         <v>1.3380000000000001</v>
       </c>
       <c r="F40" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E40</f>
         <v>2.5280061969056136</v>
       </c>
       <c r="G40" s="6">
@@ -2602,14 +2611,14 @@
         <v>194</v>
       </c>
       <c r="D41" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E41&gt;0,"Up",IF(E41&lt;0,"Down","No change"))</f>
         <v>Up</v>
       </c>
       <c r="E41" s="5">
         <v>1.726</v>
       </c>
       <c r="F41" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E41</f>
         <v>3.3080934737730625</v>
       </c>
       <c r="G41" s="6">
@@ -2639,14 +2648,14 @@
         <v>199</v>
       </c>
       <c r="D42" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E42&gt;0,"Up",IF(E42&lt;0,"Down","No change"))</f>
         <v>Up</v>
       </c>
       <c r="E42" s="5">
         <v>0.56499999999999995</v>
       </c>
       <c r="F42" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E42</f>
         <v>1.4793875092488373</v>
       </c>
       <c r="G42" s="6">
@@ -2676,14 +2685,14 @@
         <v>204</v>
       </c>
       <c r="D43" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E43&gt;0,"Up",IF(E43&lt;0,"Down","No change"))</f>
         <v>Up</v>
       </c>
       <c r="E43" s="5">
         <v>0.94799999999999995</v>
       </c>
       <c r="F43" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E43</f>
         <v>1.9291963691682765</v>
       </c>
       <c r="G43" s="6">
@@ -2713,14 +2722,14 @@
         <v>209</v>
       </c>
       <c r="D44" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E44&gt;0,"Up",IF(E44&lt;0,"Down","No change"))</f>
         <v>Up</v>
       </c>
       <c r="E44" s="5">
         <v>0.73199999999999998</v>
       </c>
       <c r="F44" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E44</f>
         <v>1.6609400481817882</v>
       </c>
       <c r="G44" s="6">
@@ -2750,14 +2759,14 @@
         <v>214</v>
       </c>
       <c r="D45" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E45&gt;0,"Up",IF(E45&lt;0,"Down","No change"))</f>
         <v>Down</v>
       </c>
       <c r="E45" s="5">
         <v>-0.36299999999999999</v>
       </c>
       <c r="F45" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E45</f>
         <v>0.77754603588255844</v>
       </c>
       <c r="G45" s="6">
@@ -2787,14 +2796,14 @@
         <v>219</v>
       </c>
       <c r="D46" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E46&gt;0,"Up",IF(E46&lt;0,"Down","No change"))</f>
         <v>Down</v>
       </c>
       <c r="E46" s="5">
         <v>-0.64100000000000001</v>
       </c>
       <c r="F46" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E46</f>
         <v>0.64126830138112412</v>
       </c>
       <c r="G46" s="6">
@@ -2824,14 +2833,14 @@
         <v>224</v>
       </c>
       <c r="D47" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E47&gt;0,"Up",IF(E47&lt;0,"Down","No change"))</f>
         <v>Down</v>
       </c>
       <c r="E47" s="5">
         <v>-0.78800000000000003</v>
       </c>
       <c r="F47" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E47</f>
         <v>0.57914640309732157</v>
       </c>
       <c r="G47" s="6">
@@ -2861,14 +2870,14 @@
         <v>229</v>
       </c>
       <c r="D48" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E48&gt;0,"Up",IF(E48&lt;0,"Down","No change"))</f>
         <v>Down</v>
       </c>
       <c r="E48" s="5">
         <v>-0.80200000000000005</v>
       </c>
       <c r="F48" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E48</f>
         <v>0.57355351211308259</v>
       </c>
       <c r="G48" s="6">
@@ -2898,14 +2907,14 @@
         <v>234</v>
       </c>
       <c r="D49" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E49&gt;0,"Up",IF(E49&lt;0,"Down","No change"))</f>
         <v>Down</v>
       </c>
       <c r="E49" s="5">
         <v>-0.81299999999999994</v>
       </c>
       <c r="F49" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E49</f>
         <v>0.56919701453743887</v>
       </c>
       <c r="G49" s="6">
@@ -2935,14 +2944,14 @@
         <v>239</v>
       </c>
       <c r="D50" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E50&gt;0,"Up",IF(E50&lt;0,"Down","No change"))</f>
         <v>Down</v>
       </c>
       <c r="E50" s="5">
         <v>-0.99299999999999999</v>
       </c>
       <c r="F50" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E50</f>
         <v>0.50243191021189282</v>
       </c>
       <c r="G50" s="6">
@@ -2972,14 +2981,14 @@
         <v>244</v>
       </c>
       <c r="D51" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E51&gt;0,"Up",IF(E51&lt;0,"Down","No change"))</f>
         <v>Up</v>
       </c>
       <c r="E51" s="5">
         <v>0.99</v>
       </c>
       <c r="F51" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E51</f>
         <v>1.9861849908740716</v>
       </c>
       <c r="G51" s="6">
@@ -3009,14 +3018,14 @@
         <v>249</v>
       </c>
       <c r="D52" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E52&gt;0,"Up",IF(E52&lt;0,"Down","No change"))</f>
         <v>Up</v>
       </c>
       <c r="E52" s="5">
         <v>0.94299999999999995</v>
       </c>
       <c r="F52" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E52</f>
         <v>1.9225218567775226</v>
       </c>
       <c r="G52" s="6">
@@ -3046,14 +3055,14 @@
         <v>254</v>
       </c>
       <c r="D53" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E53&gt;0,"Up",IF(E53&lt;0,"Down","No change"))</f>
         <v>Up</v>
       </c>
       <c r="E53" s="5">
         <v>0.91600000000000004</v>
       </c>
       <c r="F53" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E53</f>
         <v>1.8868765017907201</v>
       </c>
       <c r="G53" s="6">
@@ -3083,14 +3092,14 @@
         <v>259</v>
       </c>
       <c r="D54" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E54&gt;0,"Up",IF(E54&lt;0,"Down","No change"))</f>
         <v>Up</v>
       </c>
       <c r="E54" s="5">
         <v>1.7929999999999999</v>
       </c>
       <c r="F54" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E54</f>
         <v>3.4653474256003487</v>
       </c>
       <c r="G54" s="6">
@@ -3120,14 +3129,14 @@
         <v>263</v>
       </c>
       <c r="D55" s="4" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E55&gt;0,"Up",IF(E55&lt;0,"Down","No change"))</f>
         <v>Up</v>
       </c>
       <c r="E55" s="5">
         <v>0.59</v>
       </c>
       <c r="F55" s="5">
-        <f t="shared" si="3"/>
+        <f>2^E55</f>
         <v>1.5052467474110671</v>
       </c>
       <c r="G55" s="6">
@@ -3146,41 +3155,9 @@
         <v>265</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="64" customHeight="1">
-      <c r="A56" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>267</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>268</v>
-      </c>
-      <c r="D56" s="4" t="str">
-        <f t="shared" si="2"/>
-        <v>Up</v>
-      </c>
-      <c r="E56" s="5">
-        <v>1.327</v>
-      </c>
-      <c r="F56" s="5">
-        <f t="shared" si="3"/>
-        <v>2.5088044090419896</v>
-      </c>
-      <c r="G56" s="6">
-        <v>5.0140845070422496E-3</v>
-      </c>
-      <c r="H56" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I56" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="J56" s="4" t="s">
-        <v>269</v>
-      </c>
-      <c r="K56" s="4" t="s">
-        <v>270</v>
+    <row r="56" spans="1:11">
+      <c r="B56" t="s">
+        <v>277</v>
       </c>
     </row>
   </sheetData>
@@ -3188,16 +3165,16 @@
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G56">
-    <cfRule type="expression" dxfId="2" priority="1">
+  <conditionalFormatting sqref="G5:G55">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>G5&gt;0.05</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:H56">
-    <cfRule type="expression" dxfId="1" priority="2">
+  <conditionalFormatting sqref="H5:H55">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>H5="Very high"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>H5="Secondary"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3219,47 +3196,47 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18">
       <c r="A1" s="1" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15">
       <c r="A3" s="3" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15">
       <c r="A4" s="3" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="30">
       <c r="A5" s="3" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15">
       <c r="A6" s="3" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15">
       <c r="A7" s="3" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
     </row>
   </sheetData>

</xml_diff>